<commit_message>
Follow-on dashboard improvements: docs, finance UX, bulk ops, training UX
Update DASHBOARD, DATA_MODEL, sample import (Company_ID) and regenerate sample xlsx.
Finance: ledger filters and pagination, admin audit log viewer, invoice line editor,
refund validation (negative amount with method refund), Excel ledger export, audit GET.
Operations: bulk enrollment status update API and UI.
Training: default 1 group, single trainer share link, participant landing + Continue
before join; groups_count 1-12 in schema and migration; group picker for attendance,
attendance CSV export.
Document n8n finance snapshot and add sample workflow JSON.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/sample-import/SBS_operations_sample.xlsx
+++ b/docs/sample-import/SBS_operations_sample.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:N3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -434,12 +434,15 @@
         <v>City</v>
       </c>
       <c r="K1" t="str">
+        <v>Company_ID</v>
+      </c>
+      <c r="L1" t="str">
         <v>Created_Date</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>Status</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>Notes</v>
       </c>
     </row>
@@ -475,12 +478,15 @@
         <v>Cairo</v>
       </c>
       <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
         <v>2026-01-15</v>
       </c>
-      <c r="L2" t="str">
+      <c r="M2" t="str">
         <v>Active</v>
       </c>
-      <c r="M2" t="str">
+      <c r="N2" t="str">
         <v>Demo import row</v>
       </c>
     </row>
@@ -516,18 +522,21 @@
         <v>Alexandria</v>
       </c>
       <c r="K3" t="str">
+        <v/>
+      </c>
+      <c r="L3" t="str">
         <v>2026-02-01</v>
       </c>
-      <c r="L3" t="str">
+      <c r="M3" t="str">
         <v>Active</v>
       </c>
-      <c r="M3" t="str">
+      <c r="N3" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>